<commit_message>
chore(kmrl): synchronize approved PHY-MEC-007 binary catalog
</commit_message>
<xml_diff>
--- a/apps/kmrl-sandbox/KALP_STEM_LAB_MASTER_CATALOG_v1_0.xlsx
+++ b/apps/kmrl-sandbox/KALP_STEM_LAB_MASTER_CATALOG_v1_0.xlsx
@@ -3969,6 +3969,9 @@
       <c r="H2" t="str">
         <v>YES</v>
       </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -3995,6 +3998,9 @@
       <c r="H3" t="str">
         <v>YES</v>
       </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -4021,6 +4027,9 @@
       <c r="H4" t="str">
         <v>NO</v>
       </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -4047,6 +4056,9 @@
       <c r="H5" t="str">
         <v>YES</v>
       </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -4073,6 +4085,9 @@
       <c r="H6" t="str">
         <v>YES</v>
       </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -4099,6 +4114,9 @@
       <c r="H7" t="str">
         <v>NO</v>
       </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -4125,6 +4143,9 @@
       <c r="H8" t="str">
         <v>YES</v>
       </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -4151,6 +4172,9 @@
       <c r="H9" t="str">
         <v>YES</v>
       </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -4177,6 +4201,9 @@
       <c r="H10" t="str">
         <v>NO</v>
       </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -4203,6 +4230,9 @@
       <c r="H11" t="str">
         <v>YES</v>
       </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -4229,6 +4259,9 @@
       <c r="H12" t="str">
         <v>YES</v>
       </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -4255,6 +4288,9 @@
       <c r="H13" t="str">
         <v>NO</v>
       </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -4281,6 +4317,9 @@
       <c r="H14" t="str">
         <v>YES</v>
       </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -4307,6 +4346,9 @@
       <c r="H15" t="str">
         <v>YES</v>
       </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -4333,6 +4375,9 @@
       <c r="H16" t="str">
         <v>NO</v>
       </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -4359,6 +4404,9 @@
       <c r="H17" t="str">
         <v>YES</v>
       </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -4385,6 +4433,9 @@
       <c r="H18" t="str">
         <v>YES</v>
       </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -4411,6 +4462,9 @@
       <c r="H19" t="str">
         <v>NO</v>
       </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -4524,6 +4578,9 @@
       <c r="H23" t="str">
         <v>YES</v>
       </c>
+      <c r="I23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -4550,6 +4607,9 @@
       <c r="H24" t="str">
         <v>YES</v>
       </c>
+      <c r="I24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -4576,6 +4636,9 @@
       <c r="H25" t="str">
         <v>NO</v>
       </c>
+      <c r="I25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -4602,6 +4665,9 @@
       <c r="H26" t="str">
         <v>YES</v>
       </c>
+      <c r="I26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -4628,6 +4694,9 @@
       <c r="H27" t="str">
         <v>YES</v>
       </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -4654,6 +4723,9 @@
       <c r="H28" t="str">
         <v>NO</v>
       </c>
+      <c r="I28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -4680,6 +4752,9 @@
       <c r="H29" t="str">
         <v>YES</v>
       </c>
+      <c r="I29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -4706,6 +4781,9 @@
       <c r="H30" t="str">
         <v>YES</v>
       </c>
+      <c r="I30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -4732,6 +4810,9 @@
       <c r="H31" t="str">
         <v>NO</v>
       </c>
+      <c r="I31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -4758,6 +4839,9 @@
       <c r="H32" t="str">
         <v>YES</v>
       </c>
+      <c r="I32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -4784,6 +4868,9 @@
       <c r="H33" t="str">
         <v>YES</v>
       </c>
+      <c r="I33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -4810,6 +4897,9 @@
       <c r="H34" t="str">
         <v>NO</v>
       </c>
+      <c r="I34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -4836,6 +4926,9 @@
       <c r="H35" t="str">
         <v>YES</v>
       </c>
+      <c r="I35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -4862,6 +4955,9 @@
       <c r="H36" t="str">
         <v>YES</v>
       </c>
+      <c r="I36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -4888,6 +4984,9 @@
       <c r="H37" t="str">
         <v>NO</v>
       </c>
+      <c r="I37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -4914,6 +5013,9 @@
       <c r="H38" t="str">
         <v>YES</v>
       </c>
+      <c r="I38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -4940,6 +5042,9 @@
       <c r="H39" t="str">
         <v>YES</v>
       </c>
+      <c r="I39" t="str">
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -4966,6 +5071,9 @@
       <c r="H40" t="str">
         <v>NO</v>
       </c>
+      <c r="I40" t="str">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -4992,6 +5100,9 @@
       <c r="H41" t="str">
         <v>YES</v>
       </c>
+      <c r="I41" t="str">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -5018,6 +5129,9 @@
       <c r="H42" t="str">
         <v>YES</v>
       </c>
+      <c r="I42" t="str">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -5044,6 +5158,9 @@
       <c r="H43" t="str">
         <v>NO</v>
       </c>
+      <c r="I43" t="str">
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -5070,6 +5187,9 @@
       <c r="H44" t="str">
         <v>YES</v>
       </c>
+      <c r="I44" t="str">
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -5096,6 +5216,9 @@
       <c r="H45" t="str">
         <v>YES</v>
       </c>
+      <c r="I45" t="str">
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -5122,6 +5245,9 @@
       <c r="H46" t="str">
         <v>NO</v>
       </c>
+      <c r="I46" t="str">
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -5148,6 +5274,9 @@
       <c r="H47" t="str">
         <v>YES</v>
       </c>
+      <c r="I47" t="str">
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -5174,6 +5303,9 @@
       <c r="H48" t="str">
         <v>YES</v>
       </c>
+      <c r="I48" t="str">
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -5200,6 +5332,9 @@
       <c r="H49" t="str">
         <v>NO</v>
       </c>
+      <c r="I49" t="str">
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -5226,6 +5361,9 @@
       <c r="H50" t="str">
         <v>YES</v>
       </c>
+      <c r="I50" t="str">
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -5252,6 +5390,9 @@
       <c r="H51" t="str">
         <v>YES</v>
       </c>
+      <c r="I51" t="str">
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -5278,6 +5419,9 @@
       <c r="H52" t="str">
         <v>NO</v>
       </c>
+      <c r="I52" t="str">
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -5304,6 +5448,9 @@
       <c r="H53" t="str">
         <v>YES</v>
       </c>
+      <c r="I53" t="str">
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -5330,6 +5477,9 @@
       <c r="H54" t="str">
         <v>YES</v>
       </c>
+      <c r="I54" t="str">
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -5356,6 +5506,9 @@
       <c r="H55" t="str">
         <v>NO</v>
       </c>
+      <c r="I55" t="str">
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -5382,6 +5535,9 @@
       <c r="H56" t="str">
         <v>YES</v>
       </c>
+      <c r="I56" t="str">
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -5408,6 +5564,9 @@
       <c r="H57" t="str">
         <v>YES</v>
       </c>
+      <c r="I57" t="str">
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -5434,6 +5593,9 @@
       <c r="H58" t="str">
         <v>NO</v>
       </c>
+      <c r="I58" t="str">
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -5460,6 +5622,9 @@
       <c r="H59" t="str">
         <v>YES</v>
       </c>
+      <c r="I59" t="str">
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -5486,6 +5651,9 @@
       <c r="H60" t="str">
         <v>YES</v>
       </c>
+      <c r="I60" t="str">
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -5512,6 +5680,9 @@
       <c r="H61" t="str">
         <v>NO</v>
       </c>
+      <c r="I61" t="str">
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -5538,6 +5709,9 @@
       <c r="H62" t="str">
         <v>YES</v>
       </c>
+      <c r="I62" t="str">
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -5564,6 +5738,9 @@
       <c r="H63" t="str">
         <v>YES</v>
       </c>
+      <c r="I63" t="str">
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -5590,6 +5767,9 @@
       <c r="H64" t="str">
         <v>NO</v>
       </c>
+      <c r="I64" t="str">
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -5616,6 +5796,9 @@
       <c r="H65" t="str">
         <v>YES</v>
       </c>
+      <c r="I65" t="str">
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -5642,6 +5825,9 @@
       <c r="H66" t="str">
         <v>YES</v>
       </c>
+      <c r="I66" t="str">
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -5668,6 +5854,9 @@
       <c r="H67" t="str">
         <v>NO</v>
       </c>
+      <c r="I67" t="str">
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -5694,6 +5883,9 @@
       <c r="H68" t="str">
         <v>YES</v>
       </c>
+      <c r="I68" t="str">
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -5720,6 +5912,9 @@
       <c r="H69" t="str">
         <v>YES</v>
       </c>
+      <c r="I69" t="str">
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -5746,6 +5941,9 @@
       <c r="H70" t="str">
         <v>NO</v>
       </c>
+      <c r="I70" t="str">
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -5772,6 +5970,9 @@
       <c r="H71" t="str">
         <v>YES</v>
       </c>
+      <c r="I71" t="str">
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -5798,6 +5999,9 @@
       <c r="H72" t="str">
         <v>YES</v>
       </c>
+      <c r="I72" t="str">
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -5824,6 +6028,9 @@
       <c r="H73" t="str">
         <v>NO</v>
       </c>
+      <c r="I73" t="str">
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -5850,6 +6057,9 @@
       <c r="H74" t="str">
         <v>YES</v>
       </c>
+      <c r="I74" t="str">
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -5876,6 +6086,9 @@
       <c r="H75" t="str">
         <v>YES</v>
       </c>
+      <c r="I75" t="str">
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -5902,6 +6115,9 @@
       <c r="H76" t="str">
         <v>NO</v>
       </c>
+      <c r="I76" t="str">
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -5928,6 +6144,9 @@
       <c r="H77" t="str">
         <v>YES</v>
       </c>
+      <c r="I77" t="str">
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -5954,6 +6173,9 @@
       <c r="H78" t="str">
         <v>YES</v>
       </c>
+      <c r="I78" t="str">
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -5980,6 +6202,9 @@
       <c r="H79" t="str">
         <v>NO</v>
       </c>
+      <c r="I79" t="str">
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -6006,6 +6231,9 @@
       <c r="H80" t="str">
         <v>YES</v>
       </c>
+      <c r="I80" t="str">
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -6032,6 +6260,9 @@
       <c r="H81" t="str">
         <v>YES</v>
       </c>
+      <c r="I81" t="str">
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -6058,6 +6289,9 @@
       <c r="H82" t="str">
         <v>NO</v>
       </c>
+      <c r="I82" t="str">
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -6084,6 +6318,9 @@
       <c r="H83" t="str">
         <v>YES</v>
       </c>
+      <c r="I83" t="str">
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -6110,6 +6347,9 @@
       <c r="H84" t="str">
         <v>YES</v>
       </c>
+      <c r="I84" t="str">
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -6136,6 +6376,9 @@
       <c r="H85" t="str">
         <v>NO</v>
       </c>
+      <c r="I85" t="str">
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -6162,6 +6405,9 @@
       <c r="H86" t="str">
         <v>YES</v>
       </c>
+      <c r="I86" t="str">
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -6188,6 +6434,9 @@
       <c r="H87" t="str">
         <v>YES</v>
       </c>
+      <c r="I87" t="str">
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
@@ -6214,6 +6463,9 @@
       <c r="H88" t="str">
         <v>NO</v>
       </c>
+      <c r="I88" t="str">
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
@@ -6240,6 +6492,9 @@
       <c r="H89" t="str">
         <v>YES</v>
       </c>
+      <c r="I89" t="str">
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
@@ -6266,6 +6521,9 @@
       <c r="H90" t="str">
         <v>YES</v>
       </c>
+      <c r="I90" t="str">
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
@@ -6292,6 +6550,9 @@
       <c r="H91" t="str">
         <v>NO</v>
       </c>
+      <c r="I91" t="str">
+        <v/>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
@@ -6318,6 +6579,9 @@
       <c r="H92" t="str">
         <v>YES</v>
       </c>
+      <c r="I92" t="str">
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
@@ -6344,6 +6608,9 @@
       <c r="H93" t="str">
         <v>YES</v>
       </c>
+      <c r="I93" t="str">
+        <v/>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
@@ -6370,6 +6637,9 @@
       <c r="H94" t="str">
         <v>NO</v>
       </c>
+      <c r="I94" t="str">
+        <v/>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
@@ -6396,6 +6666,9 @@
       <c r="H95" t="str">
         <v>YES</v>
       </c>
+      <c r="I95" t="str">
+        <v/>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
@@ -6422,6 +6695,9 @@
       <c r="H96" t="str">
         <v>YES</v>
       </c>
+      <c r="I96" t="str">
+        <v/>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
@@ -6448,6 +6724,9 @@
       <c r="H97" t="str">
         <v>NO</v>
       </c>
+      <c r="I97" t="str">
+        <v/>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
@@ -6474,6 +6753,9 @@
       <c r="H98" t="str">
         <v>YES</v>
       </c>
+      <c r="I98" t="str">
+        <v/>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
@@ -6500,6 +6782,9 @@
       <c r="H99" t="str">
         <v>YES</v>
       </c>
+      <c r="I99" t="str">
+        <v/>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
@@ -6526,6 +6811,9 @@
       <c r="H100" t="str">
         <v>NO</v>
       </c>
+      <c r="I100" t="str">
+        <v/>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
@@ -6552,6 +6840,9 @@
       <c r="H101" t="str">
         <v>YES</v>
       </c>
+      <c r="I101" t="str">
+        <v/>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
@@ -6578,6 +6869,9 @@
       <c r="H102" t="str">
         <v>YES</v>
       </c>
+      <c r="I102" t="str">
+        <v/>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
@@ -6604,6 +6898,9 @@
       <c r="H103" t="str">
         <v>NO</v>
       </c>
+      <c r="I103" t="str">
+        <v/>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
@@ -6630,6 +6927,9 @@
       <c r="H104" t="str">
         <v>YES</v>
       </c>
+      <c r="I104" t="str">
+        <v/>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
@@ -6656,6 +6956,9 @@
       <c r="H105" t="str">
         <v>YES</v>
       </c>
+      <c r="I105" t="str">
+        <v/>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
@@ -6682,6 +6985,9 @@
       <c r="H106" t="str">
         <v>NO</v>
       </c>
+      <c r="I106" t="str">
+        <v/>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
@@ -6708,6 +7014,9 @@
       <c r="H107" t="str">
         <v>YES</v>
       </c>
+      <c r="I107" t="str">
+        <v/>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
@@ -6734,6 +7043,9 @@
       <c r="H108" t="str">
         <v>YES</v>
       </c>
+      <c r="I108" t="str">
+        <v/>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
@@ -6760,6 +7072,9 @@
       <c r="H109" t="str">
         <v>NO</v>
       </c>
+      <c r="I109" t="str">
+        <v/>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
@@ -6786,6 +7101,9 @@
       <c r="H110" t="str">
         <v>YES</v>
       </c>
+      <c r="I110" t="str">
+        <v/>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
@@ -6812,6 +7130,9 @@
       <c r="H111" t="str">
         <v>YES</v>
       </c>
+      <c r="I111" t="str">
+        <v/>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
@@ -6838,6 +7159,9 @@
       <c r="H112" t="str">
         <v>NO</v>
       </c>
+      <c r="I112" t="str">
+        <v/>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
@@ -6864,6 +7188,9 @@
       <c r="H113" t="str">
         <v>YES</v>
       </c>
+      <c r="I113" t="str">
+        <v/>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
@@ -6890,6 +7217,9 @@
       <c r="H114" t="str">
         <v>YES</v>
       </c>
+      <c r="I114" t="str">
+        <v/>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
@@ -6916,6 +7246,9 @@
       <c r="H115" t="str">
         <v>NO</v>
       </c>
+      <c r="I115" t="str">
+        <v/>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
@@ -6942,6 +7275,9 @@
       <c r="H116" t="str">
         <v>YES</v>
       </c>
+      <c r="I116" t="str">
+        <v/>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
@@ -6968,6 +7304,9 @@
       <c r="H117" t="str">
         <v>YES</v>
       </c>
+      <c r="I117" t="str">
+        <v/>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
@@ -6994,6 +7333,9 @@
       <c r="H118" t="str">
         <v>NO</v>
       </c>
+      <c r="I118" t="str">
+        <v/>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
@@ -7020,6 +7362,9 @@
       <c r="H119" t="str">
         <v>YES</v>
       </c>
+      <c r="I119" t="str">
+        <v/>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
@@ -7046,6 +7391,9 @@
       <c r="H120" t="str">
         <v>YES</v>
       </c>
+      <c r="I120" t="str">
+        <v/>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
@@ -7072,6 +7420,9 @@
       <c r="H121" t="str">
         <v>NO</v>
       </c>
+      <c r="I121" t="str">
+        <v/>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
@@ -7098,6 +7449,9 @@
       <c r="H122" t="str">
         <v>YES</v>
       </c>
+      <c r="I122" t="str">
+        <v/>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
@@ -7124,6 +7478,9 @@
       <c r="H123" t="str">
         <v>YES</v>
       </c>
+      <c r="I123" t="str">
+        <v/>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="str">
@@ -7150,6 +7507,9 @@
       <c r="H124" t="str">
         <v>NO</v>
       </c>
+      <c r="I124" t="str">
+        <v/>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
@@ -7176,6 +7536,9 @@
       <c r="H125" t="str">
         <v>YES</v>
       </c>
+      <c r="I125" t="str">
+        <v/>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
@@ -7202,6 +7565,9 @@
       <c r="H126" t="str">
         <v>YES</v>
       </c>
+      <c r="I126" t="str">
+        <v/>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
@@ -7228,6 +7594,9 @@
       <c r="H127" t="str">
         <v>NO</v>
       </c>
+      <c r="I127" t="str">
+        <v/>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
@@ -7254,6 +7623,9 @@
       <c r="H128" t="str">
         <v>YES</v>
       </c>
+      <c r="I128" t="str">
+        <v/>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
@@ -7280,6 +7652,9 @@
       <c r="H129" t="str">
         <v>YES</v>
       </c>
+      <c r="I129" t="str">
+        <v/>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
@@ -7306,6 +7681,9 @@
       <c r="H130" t="str">
         <v>NO</v>
       </c>
+      <c r="I130" t="str">
+        <v/>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
@@ -7332,6 +7710,9 @@
       <c r="H131" t="str">
         <v>YES</v>
       </c>
+      <c r="I131" t="str">
+        <v/>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="str">
@@ -7358,6 +7739,9 @@
       <c r="H132" t="str">
         <v>YES</v>
       </c>
+      <c r="I132" t="str">
+        <v/>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="str">
@@ -7384,6 +7768,9 @@
       <c r="H133" t="str">
         <v>NO</v>
       </c>
+      <c r="I133" t="str">
+        <v/>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="str">
@@ -7410,6 +7797,9 @@
       <c r="H134" t="str">
         <v>YES</v>
       </c>
+      <c r="I134" t="str">
+        <v/>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="str">
@@ -7436,6 +7826,9 @@
       <c r="H135" t="str">
         <v>YES</v>
       </c>
+      <c r="I135" t="str">
+        <v/>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="str">
@@ -7461,6 +7854,9 @@
       </c>
       <c r="H136" t="str">
         <v>NO</v>
+      </c>
+      <c r="I136" t="str">
+        <v/>
       </c>
     </row>
     <row r="137">
@@ -7530,7 +7926,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E181"/>
+  <dimension ref="A1:E180"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -7965,13 +8361,13 @@
         <v>1</v>
       </c>
       <c r="C26" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D26" t="str">
-        <v>Observe Conservation of Momentum</v>
+        <v>Set initial masses and velocities</v>
       </c>
       <c r="E26" t="str">
-        <v>Model/UI defined</v>
+        <v>MODEL_DEFINED</v>
       </c>
     </row>
     <row r="27">
@@ -8010,19 +8406,19 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>PHY-MEC-007</v>
+        <v>PHY-MEC-008</v>
       </c>
       <c r="B29">
         <v>1</v>
       </c>
       <c r="C29" t="str">
-        <v>INTERACT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D29" t="str">
-        <v>Set initial masses and velocities</v>
+        <v>Observe Work and Energy</v>
       </c>
       <c r="E29" t="str">
-        <v>MODEL_DEFINED</v>
+        <v>Model/UI defined</v>
       </c>
     </row>
     <row r="30">
@@ -8030,13 +8426,13 @@
         <v>PHY-MEC-008</v>
       </c>
       <c r="B30">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C30" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D30" t="str">
-        <v>Observe Work and Energy</v>
+        <v>Interact Work and Energy</v>
       </c>
       <c r="E30" t="str">
         <v>Model/UI defined</v>
@@ -8047,13 +8443,13 @@
         <v>PHY-MEC-008</v>
       </c>
       <c r="B31">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C31" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D31" t="str">
-        <v>Interact Work and Energy</v>
+        <v>Measure Work and Energy</v>
       </c>
       <c r="E31" t="str">
         <v>Model/UI defined</v>
@@ -8064,13 +8460,13 @@
         <v>PHY-MEC-008</v>
       </c>
       <c r="B32">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C32" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D32" t="str">
-        <v>Measure Work and Energy</v>
+        <v>Reflect Work and Energy</v>
       </c>
       <c r="E32" t="str">
         <v>Model/UI defined</v>
@@ -8078,16 +8474,16 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>PHY-MEC-008</v>
+        <v>PHY-MEC-009</v>
       </c>
       <c r="B33">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C33" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D33" t="str">
-        <v>Reflect Work and Energy</v>
+        <v>Observe Power Measurement</v>
       </c>
       <c r="E33" t="str">
         <v>Model/UI defined</v>
@@ -8098,13 +8494,13 @@
         <v>PHY-MEC-009</v>
       </c>
       <c r="B34">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C34" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D34" t="str">
-        <v>Observe Power Measurement</v>
+        <v>Interact Power Measurement</v>
       </c>
       <c r="E34" t="str">
         <v>Model/UI defined</v>
@@ -8115,13 +8511,13 @@
         <v>PHY-MEC-009</v>
       </c>
       <c r="B35">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C35" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D35" t="str">
-        <v>Interact Power Measurement</v>
+        <v>Measure Power Measurement</v>
       </c>
       <c r="E35" t="str">
         <v>Model/UI defined</v>
@@ -8132,13 +8528,13 @@
         <v>PHY-MEC-009</v>
       </c>
       <c r="B36">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C36" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D36" t="str">
-        <v>Measure Power Measurement</v>
+        <v>Reflect Power Measurement</v>
       </c>
       <c r="E36" t="str">
         <v>Model/UI defined</v>
@@ -8146,16 +8542,16 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>PHY-MEC-009</v>
+        <v>PHY-MEC-010</v>
       </c>
       <c r="B37">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C37" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D37" t="str">
-        <v>Reflect Power Measurement</v>
+        <v>Observe Circular Motion</v>
       </c>
       <c r="E37" t="str">
         <v>Model/UI defined</v>
@@ -8166,13 +8562,13 @@
         <v>PHY-MEC-010</v>
       </c>
       <c r="B38">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C38" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D38" t="str">
-        <v>Observe Circular Motion</v>
+        <v>Interact Circular Motion</v>
       </c>
       <c r="E38" t="str">
         <v>Model/UI defined</v>
@@ -8183,13 +8579,13 @@
         <v>PHY-MEC-010</v>
       </c>
       <c r="B39">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C39" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D39" t="str">
-        <v>Interact Circular Motion</v>
+        <v>Measure Circular Motion</v>
       </c>
       <c r="E39" t="str">
         <v>Model/UI defined</v>
@@ -8200,13 +8596,13 @@
         <v>PHY-MEC-010</v>
       </c>
       <c r="B40">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C40" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D40" t="str">
-        <v>Measure Circular Motion</v>
+        <v>Reflect Circular Motion</v>
       </c>
       <c r="E40" t="str">
         <v>Model/UI defined</v>
@@ -8214,16 +8610,16 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>PHY-MEC-010</v>
+        <v>PHY-THM-001</v>
       </c>
       <c r="B41">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C41" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D41" t="str">
-        <v>Reflect Circular Motion</v>
+        <v>Observe Heating and Cooling</v>
       </c>
       <c r="E41" t="str">
         <v>Model/UI defined</v>
@@ -8234,13 +8630,13 @@
         <v>PHY-THM-001</v>
       </c>
       <c r="B42">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C42" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D42" t="str">
-        <v>Observe Heating and Cooling</v>
+        <v>Interact Heating and Cooling</v>
       </c>
       <c r="E42" t="str">
         <v>Model/UI defined</v>
@@ -8251,13 +8647,13 @@
         <v>PHY-THM-001</v>
       </c>
       <c r="B43">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C43" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D43" t="str">
-        <v>Interact Heating and Cooling</v>
+        <v>Measure Heating and Cooling</v>
       </c>
       <c r="E43" t="str">
         <v>Model/UI defined</v>
@@ -8268,13 +8664,13 @@
         <v>PHY-THM-001</v>
       </c>
       <c r="B44">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C44" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D44" t="str">
-        <v>Measure Heating and Cooling</v>
+        <v>Reflect Heating and Cooling</v>
       </c>
       <c r="E44" t="str">
         <v>Model/UI defined</v>
@@ -8282,16 +8678,16 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>PHY-THM-001</v>
+        <v>PHY-THM-002</v>
       </c>
       <c r="B45">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C45" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D45" t="str">
-        <v>Reflect Heating and Cooling</v>
+        <v>Observe Thermal Expansion</v>
       </c>
       <c r="E45" t="str">
         <v>Model/UI defined</v>
@@ -8302,13 +8698,13 @@
         <v>PHY-THM-002</v>
       </c>
       <c r="B46">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C46" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D46" t="str">
-        <v>Observe Thermal Expansion</v>
+        <v>Interact Thermal Expansion</v>
       </c>
       <c r="E46" t="str">
         <v>Model/UI defined</v>
@@ -8319,13 +8715,13 @@
         <v>PHY-THM-002</v>
       </c>
       <c r="B47">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C47" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D47" t="str">
-        <v>Interact Thermal Expansion</v>
+        <v>Measure Thermal Expansion</v>
       </c>
       <c r="E47" t="str">
         <v>Model/UI defined</v>
@@ -8336,13 +8732,13 @@
         <v>PHY-THM-002</v>
       </c>
       <c r="B48">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C48" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D48" t="str">
-        <v>Measure Thermal Expansion</v>
+        <v>Reflect Thermal Expansion</v>
       </c>
       <c r="E48" t="str">
         <v>Model/UI defined</v>
@@ -8350,16 +8746,16 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>PHY-THM-002</v>
+        <v>PHY-OPT-001</v>
       </c>
       <c r="B49">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C49" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D49" t="str">
-        <v>Reflect Thermal Expansion</v>
+        <v>Observe Reflection from a Mirror</v>
       </c>
       <c r="E49" t="str">
         <v>Model/UI defined</v>
@@ -8370,13 +8766,13 @@
         <v>PHY-OPT-001</v>
       </c>
       <c r="B50">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C50" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D50" t="str">
-        <v>Observe Reflection from a Mirror</v>
+        <v>Interact Reflection from a Mirror</v>
       </c>
       <c r="E50" t="str">
         <v>Model/UI defined</v>
@@ -8387,13 +8783,13 @@
         <v>PHY-OPT-001</v>
       </c>
       <c r="B51">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C51" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D51" t="str">
-        <v>Interact Reflection from a Mirror</v>
+        <v>Measure Reflection from a Mirror</v>
       </c>
       <c r="E51" t="str">
         <v>Model/UI defined</v>
@@ -8404,13 +8800,13 @@
         <v>PHY-OPT-001</v>
       </c>
       <c r="B52">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C52" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D52" t="str">
-        <v>Measure Reflection from a Mirror</v>
+        <v>Reflect Reflection from a Mirror</v>
       </c>
       <c r="E52" t="str">
         <v>Model/UI defined</v>
@@ -8418,16 +8814,16 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>PHY-OPT-001</v>
+        <v>PHY-OPT-002</v>
       </c>
       <c r="B53">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C53" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D53" t="str">
-        <v>Reflect Reflection from a Mirror</v>
+        <v>Observe Refraction through a Medium</v>
       </c>
       <c r="E53" t="str">
         <v>Model/UI defined</v>
@@ -8438,13 +8834,13 @@
         <v>PHY-OPT-002</v>
       </c>
       <c r="B54">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C54" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D54" t="str">
-        <v>Observe Refraction through a Medium</v>
+        <v>Interact Refraction through a Medium</v>
       </c>
       <c r="E54" t="str">
         <v>Model/UI defined</v>
@@ -8455,13 +8851,13 @@
         <v>PHY-OPT-002</v>
       </c>
       <c r="B55">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C55" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D55" t="str">
-        <v>Interact Refraction through a Medium</v>
+        <v>Measure Refraction through a Medium</v>
       </c>
       <c r="E55" t="str">
         <v>Model/UI defined</v>
@@ -8472,13 +8868,13 @@
         <v>PHY-OPT-002</v>
       </c>
       <c r="B56">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C56" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D56" t="str">
-        <v>Measure Refraction through a Medium</v>
+        <v>Reflect Refraction through a Medium</v>
       </c>
       <c r="E56" t="str">
         <v>Model/UI defined</v>
@@ -8486,16 +8882,16 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>PHY-OPT-002</v>
+        <v>PHY-ELC-001</v>
       </c>
       <c r="B57">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C57" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D57" t="str">
-        <v>Reflect Refraction through a Medium</v>
+        <v>Observe Ohm's Law</v>
       </c>
       <c r="E57" t="str">
         <v>Model/UI defined</v>
@@ -8506,13 +8902,13 @@
         <v>PHY-ELC-001</v>
       </c>
       <c r="B58">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C58" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D58" t="str">
-        <v>Observe Ohm's Law</v>
+        <v>Interact Ohm's Law</v>
       </c>
       <c r="E58" t="str">
         <v>Model/UI defined</v>
@@ -8523,13 +8919,13 @@
         <v>PHY-ELC-001</v>
       </c>
       <c r="B59">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C59" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D59" t="str">
-        <v>Interact Ohm's Law</v>
+        <v>Measure Ohm's Law</v>
       </c>
       <c r="E59" t="str">
         <v>Model/UI defined</v>
@@ -8540,13 +8936,13 @@
         <v>PHY-ELC-001</v>
       </c>
       <c r="B60">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C60" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D60" t="str">
-        <v>Measure Ohm's Law</v>
+        <v>Reflect Ohm's Law</v>
       </c>
       <c r="E60" t="str">
         <v>Model/UI defined</v>
@@ -8554,16 +8950,16 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>PHY-ELC-001</v>
+        <v>CHE-MIX-001</v>
       </c>
       <c r="B61">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C61" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D61" t="str">
-        <v>Reflect Ohm's Law</v>
+        <v>Observe Heating Water: Observe Temperature Change</v>
       </c>
       <c r="E61" t="str">
         <v>Model/UI defined</v>
@@ -8574,13 +8970,13 @@
         <v>CHE-MIX-001</v>
       </c>
       <c r="B62">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C62" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D62" t="str">
-        <v>Observe Heating Water: Observe Temperature Change</v>
+        <v>Interact Heating Water: Observe Temperature Change</v>
       </c>
       <c r="E62" t="str">
         <v>Model/UI defined</v>
@@ -8591,13 +8987,13 @@
         <v>CHE-MIX-001</v>
       </c>
       <c r="B63">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C63" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D63" t="str">
-        <v>Interact Heating Water: Observe Temperature Change</v>
+        <v>Measure Heating Water: Observe Temperature Change</v>
       </c>
       <c r="E63" t="str">
         <v>Model/UI defined</v>
@@ -8608,13 +9004,13 @@
         <v>CHE-MIX-001</v>
       </c>
       <c r="B64">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C64" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D64" t="str">
-        <v>Measure Heating Water: Observe Temperature Change</v>
+        <v>Reflect Heating Water: Observe Temperature Change</v>
       </c>
       <c r="E64" t="str">
         <v>Model/UI defined</v>
@@ -8622,16 +9018,16 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>CHE-MIX-001</v>
+        <v>CHE-MIX-002</v>
       </c>
       <c r="B65">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C65" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D65" t="str">
-        <v>Reflect Heating Water: Observe Temperature Change</v>
+        <v>Observe Mixing Materials: Observe a System Change</v>
       </c>
       <c r="E65" t="str">
         <v>Model/UI defined</v>
@@ -8642,13 +9038,13 @@
         <v>CHE-MIX-002</v>
       </c>
       <c r="B66">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C66" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D66" t="str">
-        <v>Observe Mixing Materials: Observe a System Change</v>
+        <v>Interact Mixing Materials: Observe a System Change</v>
       </c>
       <c r="E66" t="str">
         <v>Model/UI defined</v>
@@ -8659,13 +9055,13 @@
         <v>CHE-MIX-002</v>
       </c>
       <c r="B67">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C67" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D67" t="str">
-        <v>Interact Mixing Materials: Observe a System Change</v>
+        <v>Measure Mixing Materials: Observe a System Change</v>
       </c>
       <c r="E67" t="str">
         <v>Model/UI defined</v>
@@ -8676,13 +9072,13 @@
         <v>CHE-MIX-002</v>
       </c>
       <c r="B68">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C68" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D68" t="str">
-        <v>Measure Mixing Materials: Observe a System Change</v>
+        <v>Reflect Mixing Materials: Observe a System Change</v>
       </c>
       <c r="E68" t="str">
         <v>Model/UI defined</v>
@@ -8690,16 +9086,16 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>CHE-MIX-002</v>
+        <v>CHE-ACB-001</v>
       </c>
       <c r="B69">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C69" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D69" t="str">
-        <v>Reflect Mixing Materials: Observe a System Change</v>
+        <v>Observe Acid-Base Neutralization</v>
       </c>
       <c r="E69" t="str">
         <v>Model/UI defined</v>
@@ -8710,13 +9106,13 @@
         <v>CHE-ACB-001</v>
       </c>
       <c r="B70">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C70" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D70" t="str">
-        <v>Observe Acid-Base Neutralization</v>
+        <v>Interact Acid-Base Neutralization</v>
       </c>
       <c r="E70" t="str">
         <v>Model/UI defined</v>
@@ -8727,13 +9123,13 @@
         <v>CHE-ACB-001</v>
       </c>
       <c r="B71">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C71" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D71" t="str">
-        <v>Interact Acid-Base Neutralization</v>
+        <v>Measure Acid-Base Neutralization</v>
       </c>
       <c r="E71" t="str">
         <v>Model/UI defined</v>
@@ -8744,13 +9140,13 @@
         <v>CHE-ACB-001</v>
       </c>
       <c r="B72">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C72" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D72" t="str">
-        <v>Measure Acid-Base Neutralization</v>
+        <v>Reflect Acid-Base Neutralization</v>
       </c>
       <c r="E72" t="str">
         <v>Model/UI defined</v>
@@ -8758,16 +9154,16 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>CHE-ACB-001</v>
+        <v>CHE-ACB-002</v>
       </c>
       <c r="B73">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C73" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D73" t="str">
-        <v>Reflect Acid-Base Neutralization</v>
+        <v>Observe pH and Dilution</v>
       </c>
       <c r="E73" t="str">
         <v>Model/UI defined</v>
@@ -8778,13 +9174,13 @@
         <v>CHE-ACB-002</v>
       </c>
       <c r="B74">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C74" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D74" t="str">
-        <v>Observe pH and Dilution</v>
+        <v>Interact pH and Dilution</v>
       </c>
       <c r="E74" t="str">
         <v>Model/UI defined</v>
@@ -8795,13 +9191,13 @@
         <v>CHE-ACB-002</v>
       </c>
       <c r="B75">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C75" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D75" t="str">
-        <v>Interact pH and Dilution</v>
+        <v>Measure pH and Dilution</v>
       </c>
       <c r="E75" t="str">
         <v>Model/UI defined</v>
@@ -8812,13 +9208,13 @@
         <v>CHE-ACB-002</v>
       </c>
       <c r="B76">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C76" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D76" t="str">
-        <v>Measure pH and Dilution</v>
+        <v>Reflect pH and Dilution</v>
       </c>
       <c r="E76" t="str">
         <v>Model/UI defined</v>
@@ -8826,16 +9222,16 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>CHE-ACB-002</v>
+        <v>CHE-STO-001</v>
       </c>
       <c r="B77">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C77" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D77" t="str">
-        <v>Reflect pH and Dilution</v>
+        <v>Observe Stoichiometry</v>
       </c>
       <c r="E77" t="str">
         <v>Model/UI defined</v>
@@ -8846,13 +9242,13 @@
         <v>CHE-STO-001</v>
       </c>
       <c r="B78">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C78" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D78" t="str">
-        <v>Observe Stoichiometry</v>
+        <v>Interact Stoichiometry</v>
       </c>
       <c r="E78" t="str">
         <v>Model/UI defined</v>
@@ -8863,13 +9259,13 @@
         <v>CHE-STO-001</v>
       </c>
       <c r="B79">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C79" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D79" t="str">
-        <v>Interact Stoichiometry</v>
+        <v>Measure Stoichiometry</v>
       </c>
       <c r="E79" t="str">
         <v>Model/UI defined</v>
@@ -8880,13 +9276,13 @@
         <v>CHE-STO-001</v>
       </c>
       <c r="B80">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C80" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D80" t="str">
-        <v>Measure Stoichiometry</v>
+        <v>Reflect Stoichiometry</v>
       </c>
       <c r="E80" t="str">
         <v>Model/UI defined</v>
@@ -8894,16 +9290,16 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>CHE-STO-001</v>
+        <v>CHE-STO-002</v>
       </c>
       <c r="B81">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C81" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D81" t="str">
-        <v>Reflect Stoichiometry</v>
+        <v>Observe Limiting Reagent</v>
       </c>
       <c r="E81" t="str">
         <v>Model/UI defined</v>
@@ -8914,13 +9310,13 @@
         <v>CHE-STO-002</v>
       </c>
       <c r="B82">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C82" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D82" t="str">
-        <v>Observe Limiting Reagent</v>
+        <v>Interact Limiting Reagent</v>
       </c>
       <c r="E82" t="str">
         <v>Model/UI defined</v>
@@ -8931,13 +9327,13 @@
         <v>CHE-STO-002</v>
       </c>
       <c r="B83">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C83" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D83" t="str">
-        <v>Interact Limiting Reagent</v>
+        <v>Measure Limiting Reagent</v>
       </c>
       <c r="E83" t="str">
         <v>Model/UI defined</v>
@@ -8948,13 +9344,13 @@
         <v>CHE-STO-002</v>
       </c>
       <c r="B84">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C84" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D84" t="str">
-        <v>Measure Limiting Reagent</v>
+        <v>Reflect Limiting Reagent</v>
       </c>
       <c r="E84" t="str">
         <v>Model/UI defined</v>
@@ -8962,16 +9358,16 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>CHE-STO-002</v>
+        <v>CHE-ELC-001</v>
       </c>
       <c r="B85">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C85" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D85" t="str">
-        <v>Reflect Limiting Reagent</v>
+        <v>Observe Simple Electrolysis</v>
       </c>
       <c r="E85" t="str">
         <v>Model/UI defined</v>
@@ -8982,13 +9378,13 @@
         <v>CHE-ELC-001</v>
       </c>
       <c r="B86">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C86" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D86" t="str">
-        <v>Observe Simple Electrolysis</v>
+        <v>Interact Simple Electrolysis</v>
       </c>
       <c r="E86" t="str">
         <v>Model/UI defined</v>
@@ -8999,13 +9395,13 @@
         <v>CHE-ELC-001</v>
       </c>
       <c r="B87">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C87" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D87" t="str">
-        <v>Interact Simple Electrolysis</v>
+        <v>Measure Simple Electrolysis</v>
       </c>
       <c r="E87" t="str">
         <v>Model/UI defined</v>
@@ -9016,13 +9412,13 @@
         <v>CHE-ELC-001</v>
       </c>
       <c r="B88">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C88" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D88" t="str">
-        <v>Measure Simple Electrolysis</v>
+        <v>Reflect Simple Electrolysis</v>
       </c>
       <c r="E88" t="str">
         <v>Model/UI defined</v>
@@ -9030,16 +9426,16 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>CHE-ELC-001</v>
+        <v>CHE-ELC-002</v>
       </c>
       <c r="B89">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C89" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D89" t="str">
-        <v>Reflect Simple Electrolysis</v>
+        <v>Observe Galvanic Cell</v>
       </c>
       <c r="E89" t="str">
         <v>Model/UI defined</v>
@@ -9050,13 +9446,13 @@
         <v>CHE-ELC-002</v>
       </c>
       <c r="B90">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C90" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D90" t="str">
-        <v>Observe Galvanic Cell</v>
+        <v>Interact Galvanic Cell</v>
       </c>
       <c r="E90" t="str">
         <v>Model/UI defined</v>
@@ -9067,13 +9463,13 @@
         <v>CHE-ELC-002</v>
       </c>
       <c r="B91">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C91" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D91" t="str">
-        <v>Interact Galvanic Cell</v>
+        <v>Measure Galvanic Cell</v>
       </c>
       <c r="E91" t="str">
         <v>Model/UI defined</v>
@@ -9084,13 +9480,13 @@
         <v>CHE-ELC-002</v>
       </c>
       <c r="B92">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C92" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D92" t="str">
-        <v>Measure Galvanic Cell</v>
+        <v>Reflect Galvanic Cell</v>
       </c>
       <c r="E92" t="str">
         <v>Model/UI defined</v>
@@ -9098,16 +9494,16 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>CHE-ELC-002</v>
+        <v>CHE-THM-001</v>
       </c>
       <c r="B93">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C93" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D93" t="str">
-        <v>Reflect Galvanic Cell</v>
+        <v>Observe Exothermic Reaction</v>
       </c>
       <c r="E93" t="str">
         <v>Model/UI defined</v>
@@ -9118,13 +9514,13 @@
         <v>CHE-THM-001</v>
       </c>
       <c r="B94">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C94" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D94" t="str">
-        <v>Observe Exothermic Reaction</v>
+        <v>Interact Exothermic Reaction</v>
       </c>
       <c r="E94" t="str">
         <v>Model/UI defined</v>
@@ -9135,13 +9531,13 @@
         <v>CHE-THM-001</v>
       </c>
       <c r="B95">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C95" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D95" t="str">
-        <v>Interact Exothermic Reaction</v>
+        <v>Measure Exothermic Reaction</v>
       </c>
       <c r="E95" t="str">
         <v>Model/UI defined</v>
@@ -9152,13 +9548,13 @@
         <v>CHE-THM-001</v>
       </c>
       <c r="B96">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C96" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D96" t="str">
-        <v>Measure Exothermic Reaction</v>
+        <v>Reflect Exothermic Reaction</v>
       </c>
       <c r="E96" t="str">
         <v>Model/UI defined</v>
@@ -9166,16 +9562,16 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>CHE-THM-001</v>
+        <v>CHE-THM-002</v>
       </c>
       <c r="B97">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C97" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D97" t="str">
-        <v>Reflect Exothermic Reaction</v>
+        <v>Observe Endothermic Reaction</v>
       </c>
       <c r="E97" t="str">
         <v>Model/UI defined</v>
@@ -9186,13 +9582,13 @@
         <v>CHE-THM-002</v>
       </c>
       <c r="B98">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C98" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D98" t="str">
-        <v>Observe Endothermic Reaction</v>
+        <v>Interact Endothermic Reaction</v>
       </c>
       <c r="E98" t="str">
         <v>Model/UI defined</v>
@@ -9203,13 +9599,13 @@
         <v>CHE-THM-002</v>
       </c>
       <c r="B99">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C99" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D99" t="str">
-        <v>Interact Endothermic Reaction</v>
+        <v>Measure Endothermic Reaction</v>
       </c>
       <c r="E99" t="str">
         <v>Model/UI defined</v>
@@ -9220,13 +9616,13 @@
         <v>CHE-THM-002</v>
       </c>
       <c r="B100">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C100" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D100" t="str">
-        <v>Measure Endothermic Reaction</v>
+        <v>Reflect Endothermic Reaction</v>
       </c>
       <c r="E100" t="str">
         <v>Model/UI defined</v>
@@ -9234,16 +9630,16 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>CHE-THM-002</v>
+        <v>CHE-MAT-001</v>
       </c>
       <c r="B101">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C101" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D101" t="str">
-        <v>Reflect Endothermic Reaction</v>
+        <v>Observe Steel Making</v>
       </c>
       <c r="E101" t="str">
         <v>Model/UI defined</v>
@@ -9254,13 +9650,13 @@
         <v>CHE-MAT-001</v>
       </c>
       <c r="B102">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C102" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D102" t="str">
-        <v>Observe Steel Making</v>
+        <v>Interact Steel Making</v>
       </c>
       <c r="E102" t="str">
         <v>Model/UI defined</v>
@@ -9271,13 +9667,13 @@
         <v>CHE-MAT-001</v>
       </c>
       <c r="B103">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C103" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D103" t="str">
-        <v>Interact Steel Making</v>
+        <v>Measure Steel Making</v>
       </c>
       <c r="E103" t="str">
         <v>Model/UI defined</v>
@@ -9288,13 +9684,13 @@
         <v>CHE-MAT-001</v>
       </c>
       <c r="B104">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C104" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D104" t="str">
-        <v>Measure Steel Making</v>
+        <v>Reflect Steel Making</v>
       </c>
       <c r="E104" t="str">
         <v>Model/UI defined</v>
@@ -9302,16 +9698,16 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>CHE-MAT-001</v>
+        <v>CHE-MAT-002</v>
       </c>
       <c r="B105">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C105" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D105" t="str">
-        <v>Reflect Steel Making</v>
+        <v>Observe Alloy Composition</v>
       </c>
       <c r="E105" t="str">
         <v>Model/UI defined</v>
@@ -9322,13 +9718,13 @@
         <v>CHE-MAT-002</v>
       </c>
       <c r="B106">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C106" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D106" t="str">
-        <v>Observe Alloy Composition</v>
+        <v>Interact Alloy Composition</v>
       </c>
       <c r="E106" t="str">
         <v>Model/UI defined</v>
@@ -9339,13 +9735,13 @@
         <v>CHE-MAT-002</v>
       </c>
       <c r="B107">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C107" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D107" t="str">
-        <v>Interact Alloy Composition</v>
+        <v>Measure Alloy Composition</v>
       </c>
       <c r="E107" t="str">
         <v>Model/UI defined</v>
@@ -9356,13 +9752,13 @@
         <v>CHE-MAT-002</v>
       </c>
       <c r="B108">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C108" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D108" t="str">
-        <v>Measure Alloy Composition</v>
+        <v>Reflect Alloy Composition</v>
       </c>
       <c r="E108" t="str">
         <v>Model/UI defined</v>
@@ -9370,16 +9766,16 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>CHE-MAT-002</v>
+        <v>CHE-KIN-001</v>
       </c>
       <c r="B109">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C109" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D109" t="str">
-        <v>Reflect Alloy Composition</v>
+        <v>Observe Reaction Rate vs Temperature</v>
       </c>
       <c r="E109" t="str">
         <v>Model/UI defined</v>
@@ -9390,13 +9786,13 @@
         <v>CHE-KIN-001</v>
       </c>
       <c r="B110">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C110" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D110" t="str">
-        <v>Observe Reaction Rate vs Temperature</v>
+        <v>Interact Reaction Rate vs Temperature</v>
       </c>
       <c r="E110" t="str">
         <v>Model/UI defined</v>
@@ -9407,13 +9803,13 @@
         <v>CHE-KIN-001</v>
       </c>
       <c r="B111">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C111" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D111" t="str">
-        <v>Interact Reaction Rate vs Temperature</v>
+        <v>Measure Reaction Rate vs Temperature</v>
       </c>
       <c r="E111" t="str">
         <v>Model/UI defined</v>
@@ -9424,13 +9820,13 @@
         <v>CHE-KIN-001</v>
       </c>
       <c r="B112">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C112" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D112" t="str">
-        <v>Measure Reaction Rate vs Temperature</v>
+        <v>Reflect Reaction Rate vs Temperature</v>
       </c>
       <c r="E112" t="str">
         <v>Model/UI defined</v>
@@ -9438,16 +9834,16 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>CHE-KIN-001</v>
+        <v>CHE-KIN-002</v>
       </c>
       <c r="B113">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C113" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D113" t="str">
-        <v>Reflect Reaction Rate vs Temperature</v>
+        <v>Observe Concentration and Reaction Rate</v>
       </c>
       <c r="E113" t="str">
         <v>Model/UI defined</v>
@@ -9458,13 +9854,13 @@
         <v>CHE-KIN-002</v>
       </c>
       <c r="B114">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C114" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D114" t="str">
-        <v>Observe Concentration and Reaction Rate</v>
+        <v>Interact Concentration and Reaction Rate</v>
       </c>
       <c r="E114" t="str">
         <v>Model/UI defined</v>
@@ -9475,13 +9871,13 @@
         <v>CHE-KIN-002</v>
       </c>
       <c r="B115">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C115" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D115" t="str">
-        <v>Interact Concentration and Reaction Rate</v>
+        <v>Measure Concentration and Reaction Rate</v>
       </c>
       <c r="E115" t="str">
         <v>Model/UI defined</v>
@@ -9492,13 +9888,13 @@
         <v>CHE-KIN-002</v>
       </c>
       <c r="B116">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C116" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D116" t="str">
-        <v>Measure Concentration and Reaction Rate</v>
+        <v>Reflect Concentration and Reaction Rate</v>
       </c>
       <c r="E116" t="str">
         <v>Model/UI defined</v>
@@ -9506,16 +9902,16 @@
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>CHE-KIN-002</v>
+        <v>CHE-ORG-001</v>
       </c>
       <c r="B117">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C117" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D117" t="str">
-        <v>Reflect Concentration and Reaction Rate</v>
+        <v>Observe Esterification Model</v>
       </c>
       <c r="E117" t="str">
         <v>Model/UI defined</v>
@@ -9526,13 +9922,13 @@
         <v>CHE-ORG-001</v>
       </c>
       <c r="B118">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C118" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D118" t="str">
-        <v>Observe Esterification Model</v>
+        <v>Interact Esterification Model</v>
       </c>
       <c r="E118" t="str">
         <v>Model/UI defined</v>
@@ -9543,13 +9939,13 @@
         <v>CHE-ORG-001</v>
       </c>
       <c r="B119">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C119" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D119" t="str">
-        <v>Interact Esterification Model</v>
+        <v>Measure Esterification Model</v>
       </c>
       <c r="E119" t="str">
         <v>Model/UI defined</v>
@@ -9560,13 +9956,13 @@
         <v>CHE-ORG-001</v>
       </c>
       <c r="B120">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C120" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D120" t="str">
-        <v>Measure Esterification Model</v>
+        <v>Reflect Esterification Model</v>
       </c>
       <c r="E120" t="str">
         <v>Model/UI defined</v>
@@ -9574,16 +9970,16 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>CHE-ORG-001</v>
+        <v>MAT-ALG-001</v>
       </c>
       <c r="B121">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C121" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D121" t="str">
-        <v>Reflect Esterification Model</v>
+        <v>Observe Linear Equation Lab</v>
       </c>
       <c r="E121" t="str">
         <v>Model/UI defined</v>
@@ -9594,13 +9990,13 @@
         <v>MAT-ALG-001</v>
       </c>
       <c r="B122">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C122" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D122" t="str">
-        <v>Observe Linear Equation Lab</v>
+        <v>Interact Linear Equation Lab</v>
       </c>
       <c r="E122" t="str">
         <v>Model/UI defined</v>
@@ -9611,13 +10007,13 @@
         <v>MAT-ALG-001</v>
       </c>
       <c r="B123">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C123" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D123" t="str">
-        <v>Interact Linear Equation Lab</v>
+        <v>Measure Linear Equation Lab</v>
       </c>
       <c r="E123" t="str">
         <v>Model/UI defined</v>
@@ -9628,13 +10024,13 @@
         <v>MAT-ALG-001</v>
       </c>
       <c r="B124">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C124" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D124" t="str">
-        <v>Measure Linear Equation Lab</v>
+        <v>Reflect Linear Equation Lab</v>
       </c>
       <c r="E124" t="str">
         <v>Model/UI defined</v>
@@ -9642,16 +10038,16 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>MAT-ALG-001</v>
+        <v>MAT-ALG-002</v>
       </c>
       <c r="B125">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C125" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D125" t="str">
-        <v>Reflect Linear Equation Lab</v>
+        <v>Observe Quadratic Equation Lab</v>
       </c>
       <c r="E125" t="str">
         <v>Model/UI defined</v>
@@ -9662,13 +10058,13 @@
         <v>MAT-ALG-002</v>
       </c>
       <c r="B126">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C126" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D126" t="str">
-        <v>Observe Quadratic Equation Lab</v>
+        <v>Interact Quadratic Equation Lab</v>
       </c>
       <c r="E126" t="str">
         <v>Model/UI defined</v>
@@ -9679,13 +10075,13 @@
         <v>MAT-ALG-002</v>
       </c>
       <c r="B127">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C127" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D127" t="str">
-        <v>Interact Quadratic Equation Lab</v>
+        <v>Measure Quadratic Equation Lab</v>
       </c>
       <c r="E127" t="str">
         <v>Model/UI defined</v>
@@ -9696,13 +10092,13 @@
         <v>MAT-ALG-002</v>
       </c>
       <c r="B128">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C128" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D128" t="str">
-        <v>Measure Quadratic Equation Lab</v>
+        <v>Reflect Quadratic Equation Lab</v>
       </c>
       <c r="E128" t="str">
         <v>Model/UI defined</v>
@@ -9710,16 +10106,16 @@
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>MAT-ALG-002</v>
+        <v>MAT-ALG-003</v>
       </c>
       <c r="B129">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C129" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D129" t="str">
-        <v>Reflect Quadratic Equation Lab</v>
+        <v>Observe Systems of Equations</v>
       </c>
       <c r="E129" t="str">
         <v>Model/UI defined</v>
@@ -9730,13 +10126,13 @@
         <v>MAT-ALG-003</v>
       </c>
       <c r="B130">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C130" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D130" t="str">
-        <v>Observe Systems of Equations</v>
+        <v>Interact Systems of Equations</v>
       </c>
       <c r="E130" t="str">
         <v>Model/UI defined</v>
@@ -9747,13 +10143,13 @@
         <v>MAT-ALG-003</v>
       </c>
       <c r="B131">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C131" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D131" t="str">
-        <v>Interact Systems of Equations</v>
+        <v>Measure Systems of Equations</v>
       </c>
       <c r="E131" t="str">
         <v>Model/UI defined</v>
@@ -9764,13 +10160,13 @@
         <v>MAT-ALG-003</v>
       </c>
       <c r="B132">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C132" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D132" t="str">
-        <v>Measure Systems of Equations</v>
+        <v>Reflect Systems of Equations</v>
       </c>
       <c r="E132" t="str">
         <v>Model/UI defined</v>
@@ -9778,16 +10174,16 @@
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>MAT-ALG-003</v>
+        <v>MAT-GEO-001</v>
       </c>
       <c r="B133">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C133" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D133" t="str">
-        <v>Reflect Systems of Equations</v>
+        <v>Observe Triangle Geometry</v>
       </c>
       <c r="E133" t="str">
         <v>Model/UI defined</v>
@@ -9798,13 +10194,13 @@
         <v>MAT-GEO-001</v>
       </c>
       <c r="B134">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C134" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D134" t="str">
-        <v>Observe Triangle Geometry</v>
+        <v>Interact Triangle Geometry</v>
       </c>
       <c r="E134" t="str">
         <v>Model/UI defined</v>
@@ -9815,13 +10211,13 @@
         <v>MAT-GEO-001</v>
       </c>
       <c r="B135">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C135" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D135" t="str">
-        <v>Interact Triangle Geometry</v>
+        <v>Measure Triangle Geometry</v>
       </c>
       <c r="E135" t="str">
         <v>Model/UI defined</v>
@@ -9832,13 +10228,13 @@
         <v>MAT-GEO-001</v>
       </c>
       <c r="B136">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C136" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D136" t="str">
-        <v>Measure Triangle Geometry</v>
+        <v>Reflect Triangle Geometry</v>
       </c>
       <c r="E136" t="str">
         <v>Model/UI defined</v>
@@ -9846,16 +10242,16 @@
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>MAT-GEO-001</v>
+        <v>MAT-GEO-002</v>
       </c>
       <c r="B137">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C137" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D137" t="str">
-        <v>Reflect Triangle Geometry</v>
+        <v>Observe Circle Geometry</v>
       </c>
       <c r="E137" t="str">
         <v>Model/UI defined</v>
@@ -9866,13 +10262,13 @@
         <v>MAT-GEO-002</v>
       </c>
       <c r="B138">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C138" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D138" t="str">
-        <v>Observe Circle Geometry</v>
+        <v>Interact Circle Geometry</v>
       </c>
       <c r="E138" t="str">
         <v>Model/UI defined</v>
@@ -9883,13 +10279,13 @@
         <v>MAT-GEO-002</v>
       </c>
       <c r="B139">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C139" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D139" t="str">
-        <v>Interact Circle Geometry</v>
+        <v>Measure Circle Geometry</v>
       </c>
       <c r="E139" t="str">
         <v>Model/UI defined</v>
@@ -9900,13 +10296,13 @@
         <v>MAT-GEO-002</v>
       </c>
       <c r="B140">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C140" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D140" t="str">
-        <v>Measure Circle Geometry</v>
+        <v>Reflect Circle Geometry</v>
       </c>
       <c r="E140" t="str">
         <v>Model/UI defined</v>
@@ -9914,16 +10310,16 @@
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>MAT-GEO-002</v>
+        <v>MAT-GEO-003</v>
       </c>
       <c r="B141">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C141" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D141" t="str">
-        <v>Reflect Circle Geometry</v>
+        <v>Observe Area and Volume</v>
       </c>
       <c r="E141" t="str">
         <v>Model/UI defined</v>
@@ -9934,13 +10330,13 @@
         <v>MAT-GEO-003</v>
       </c>
       <c r="B142">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C142" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D142" t="str">
-        <v>Observe Area and Volume</v>
+        <v>Interact Area and Volume</v>
       </c>
       <c r="E142" t="str">
         <v>Model/UI defined</v>
@@ -9951,13 +10347,13 @@
         <v>MAT-GEO-003</v>
       </c>
       <c r="B143">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C143" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D143" t="str">
-        <v>Interact Area and Volume</v>
+        <v>Measure Area and Volume</v>
       </c>
       <c r="E143" t="str">
         <v>Model/UI defined</v>
@@ -9968,13 +10364,13 @@
         <v>MAT-GEO-003</v>
       </c>
       <c r="B144">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C144" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D144" t="str">
-        <v>Measure Area and Volume</v>
+        <v>Reflect Area and Volume</v>
       </c>
       <c r="E144" t="str">
         <v>Model/UI defined</v>
@@ -9982,16 +10378,16 @@
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>MAT-GEO-003</v>
+        <v>MAT-TRG-001</v>
       </c>
       <c r="B145">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C145" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D145" t="str">
-        <v>Reflect Area and Volume</v>
+        <v>Observe Sine and Cosine Lab</v>
       </c>
       <c r="E145" t="str">
         <v>Model/UI defined</v>
@@ -10002,13 +10398,13 @@
         <v>MAT-TRG-001</v>
       </c>
       <c r="B146">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C146" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D146" t="str">
-        <v>Observe Sine and Cosine Lab</v>
+        <v>Interact Sine and Cosine Lab</v>
       </c>
       <c r="E146" t="str">
         <v>Model/UI defined</v>
@@ -10019,13 +10415,13 @@
         <v>MAT-TRG-001</v>
       </c>
       <c r="B147">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C147" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D147" t="str">
-        <v>Interact Sine and Cosine Lab</v>
+        <v>Measure Sine and Cosine Lab</v>
       </c>
       <c r="E147" t="str">
         <v>Model/UI defined</v>
@@ -10036,13 +10432,13 @@
         <v>MAT-TRG-001</v>
       </c>
       <c r="B148">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C148" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D148" t="str">
-        <v>Measure Sine and Cosine Lab</v>
+        <v>Reflect Sine and Cosine Lab</v>
       </c>
       <c r="E148" t="str">
         <v>Model/UI defined</v>
@@ -10050,16 +10446,16 @@
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>MAT-TRG-001</v>
+        <v>MAT-TRG-002</v>
       </c>
       <c r="B149">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C149" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D149" t="str">
-        <v>Reflect Sine and Cosine Lab</v>
+        <v>Observe Right Triangle Explorer</v>
       </c>
       <c r="E149" t="str">
         <v>Model/UI defined</v>
@@ -10070,13 +10466,13 @@
         <v>MAT-TRG-002</v>
       </c>
       <c r="B150">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C150" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D150" t="str">
-        <v>Observe Right Triangle Explorer</v>
+        <v>Interact Right Triangle Explorer</v>
       </c>
       <c r="E150" t="str">
         <v>Model/UI defined</v>
@@ -10087,13 +10483,13 @@
         <v>MAT-TRG-002</v>
       </c>
       <c r="B151">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C151" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D151" t="str">
-        <v>Interact Right Triangle Explorer</v>
+        <v>Measure Right Triangle Explorer</v>
       </c>
       <c r="E151" t="str">
         <v>Model/UI defined</v>
@@ -10104,13 +10500,13 @@
         <v>MAT-TRG-002</v>
       </c>
       <c r="B152">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C152" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D152" t="str">
-        <v>Measure Right Triangle Explorer</v>
+        <v>Reflect Right Triangle Explorer</v>
       </c>
       <c r="E152" t="str">
         <v>Model/UI defined</v>
@@ -10118,16 +10514,16 @@
     </row>
     <row r="153">
       <c r="A153" t="str">
-        <v>MAT-TRG-002</v>
+        <v>MAT-CAL-001</v>
       </c>
       <c r="B153">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C153" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D153" t="str">
-        <v>Reflect Right Triangle Explorer</v>
+        <v>Observe Derivative Explorer</v>
       </c>
       <c r="E153" t="str">
         <v>Model/UI defined</v>
@@ -10138,13 +10534,13 @@
         <v>MAT-CAL-001</v>
       </c>
       <c r="B154">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C154" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D154" t="str">
-        <v>Observe Derivative Explorer</v>
+        <v>Interact Derivative Explorer</v>
       </c>
       <c r="E154" t="str">
         <v>Model/UI defined</v>
@@ -10155,13 +10551,13 @@
         <v>MAT-CAL-001</v>
       </c>
       <c r="B155">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C155" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D155" t="str">
-        <v>Interact Derivative Explorer</v>
+        <v>Measure Derivative Explorer</v>
       </c>
       <c r="E155" t="str">
         <v>Model/UI defined</v>
@@ -10172,13 +10568,13 @@
         <v>MAT-CAL-001</v>
       </c>
       <c r="B156">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C156" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D156" t="str">
-        <v>Measure Derivative Explorer</v>
+        <v>Reflect Derivative Explorer</v>
       </c>
       <c r="E156" t="str">
         <v>Model/UI defined</v>
@@ -10186,16 +10582,16 @@
     </row>
     <row r="157">
       <c r="A157" t="str">
-        <v>MAT-CAL-001</v>
+        <v>MAT-CAL-002</v>
       </c>
       <c r="B157">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C157" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D157" t="str">
-        <v>Reflect Derivative Explorer</v>
+        <v>Observe Integral / Area Explorer</v>
       </c>
       <c r="E157" t="str">
         <v>Model/UI defined</v>
@@ -10206,13 +10602,13 @@
         <v>MAT-CAL-002</v>
       </c>
       <c r="B158">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C158" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D158" t="str">
-        <v>Observe Integral / Area Explorer</v>
+        <v>Interact Integral / Area Explorer</v>
       </c>
       <c r="E158" t="str">
         <v>Model/UI defined</v>
@@ -10223,13 +10619,13 @@
         <v>MAT-CAL-002</v>
       </c>
       <c r="B159">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C159" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D159" t="str">
-        <v>Interact Integral / Area Explorer</v>
+        <v>Measure Integral / Area Explorer</v>
       </c>
       <c r="E159" t="str">
         <v>Model/UI defined</v>
@@ -10240,13 +10636,13 @@
         <v>MAT-CAL-002</v>
       </c>
       <c r="B160">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C160" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D160" t="str">
-        <v>Measure Integral / Area Explorer</v>
+        <v>Reflect Integral / Area Explorer</v>
       </c>
       <c r="E160" t="str">
         <v>Model/UI defined</v>
@@ -10254,16 +10650,16 @@
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>MAT-CAL-002</v>
+        <v>MAT-STA-001</v>
       </c>
       <c r="B161">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C161" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D161" t="str">
-        <v>Reflect Integral / Area Explorer</v>
+        <v>Observe Mean Median Mode Lab</v>
       </c>
       <c r="E161" t="str">
         <v>Model/UI defined</v>
@@ -10274,13 +10670,13 @@
         <v>MAT-STA-001</v>
       </c>
       <c r="B162">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C162" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D162" t="str">
-        <v>Observe Mean Median Mode Lab</v>
+        <v>Interact Mean Median Mode Lab</v>
       </c>
       <c r="E162" t="str">
         <v>Model/UI defined</v>
@@ -10291,13 +10687,13 @@
         <v>MAT-STA-001</v>
       </c>
       <c r="B163">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C163" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D163" t="str">
-        <v>Interact Mean Median Mode Lab</v>
+        <v>Measure Mean Median Mode Lab</v>
       </c>
       <c r="E163" t="str">
         <v>Model/UI defined</v>
@@ -10308,13 +10704,13 @@
         <v>MAT-STA-001</v>
       </c>
       <c r="B164">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C164" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D164" t="str">
-        <v>Measure Mean Median Mode Lab</v>
+        <v>Reflect Mean Median Mode Lab</v>
       </c>
       <c r="E164" t="str">
         <v>Model/UI defined</v>
@@ -10322,16 +10718,16 @@
     </row>
     <row r="165">
       <c r="A165" t="str">
-        <v>MAT-STA-001</v>
+        <v>MAT-STA-002</v>
       </c>
       <c r="B165">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C165" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D165" t="str">
-        <v>Reflect Mean Median Mode Lab</v>
+        <v>Observe Standard Deviation Lab</v>
       </c>
       <c r="E165" t="str">
         <v>Model/UI defined</v>
@@ -10342,13 +10738,13 @@
         <v>MAT-STA-002</v>
       </c>
       <c r="B166">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C166" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D166" t="str">
-        <v>Observe Standard Deviation Lab</v>
+        <v>Interact Standard Deviation Lab</v>
       </c>
       <c r="E166" t="str">
         <v>Model/UI defined</v>
@@ -10359,13 +10755,13 @@
         <v>MAT-STA-002</v>
       </c>
       <c r="B167">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C167" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D167" t="str">
-        <v>Interact Standard Deviation Lab</v>
+        <v>Measure Standard Deviation Lab</v>
       </c>
       <c r="E167" t="str">
         <v>Model/UI defined</v>
@@ -10376,13 +10772,13 @@
         <v>MAT-STA-002</v>
       </c>
       <c r="B168">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C168" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D168" t="str">
-        <v>Measure Standard Deviation Lab</v>
+        <v>Reflect Standard Deviation Lab</v>
       </c>
       <c r="E168" t="str">
         <v>Model/UI defined</v>
@@ -10390,16 +10786,16 @@
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v>MAT-STA-002</v>
+        <v>MAT-PRB-001</v>
       </c>
       <c r="B169">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C169" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D169" t="str">
-        <v>Reflect Standard Deviation Lab</v>
+        <v>Observe Probability Simulator</v>
       </c>
       <c r="E169" t="str">
         <v>Model/UI defined</v>
@@ -10410,13 +10806,13 @@
         <v>MAT-PRB-001</v>
       </c>
       <c r="B170">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C170" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D170" t="str">
-        <v>Observe Probability Simulator</v>
+        <v>Interact Probability Simulator</v>
       </c>
       <c r="E170" t="str">
         <v>Model/UI defined</v>
@@ -10427,13 +10823,13 @@
         <v>MAT-PRB-001</v>
       </c>
       <c r="B171">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C171" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D171" t="str">
-        <v>Interact Probability Simulator</v>
+        <v>Measure Probability Simulator</v>
       </c>
       <c r="E171" t="str">
         <v>Model/UI defined</v>
@@ -10444,13 +10840,13 @@
         <v>MAT-PRB-001</v>
       </c>
       <c r="B172">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C172" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D172" t="str">
-        <v>Measure Probability Simulator</v>
+        <v>Reflect Probability Simulator</v>
       </c>
       <c r="E172" t="str">
         <v>Model/UI defined</v>
@@ -10458,16 +10854,16 @@
     </row>
     <row r="173">
       <c r="A173" t="str">
-        <v>MAT-PRB-001</v>
+        <v>MAT-VEC-001</v>
       </c>
       <c r="B173">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C173" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D173" t="str">
-        <v>Reflect Probability Simulator</v>
+        <v>Observe Vector Addition</v>
       </c>
       <c r="E173" t="str">
         <v>Model/UI defined</v>
@@ -10478,13 +10874,13 @@
         <v>MAT-VEC-001</v>
       </c>
       <c r="B174">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C174" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D174" t="str">
-        <v>Observe Vector Addition</v>
+        <v>Interact Vector Addition</v>
       </c>
       <c r="E174" t="str">
         <v>Model/UI defined</v>
@@ -10495,13 +10891,13 @@
         <v>MAT-VEC-001</v>
       </c>
       <c r="B175">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C175" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D175" t="str">
-        <v>Interact Vector Addition</v>
+        <v>Measure Vector Addition</v>
       </c>
       <c r="E175" t="str">
         <v>Model/UI defined</v>
@@ -10512,13 +10908,13 @@
         <v>MAT-VEC-001</v>
       </c>
       <c r="B176">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C176" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D176" t="str">
-        <v>Measure Vector Addition</v>
+        <v>Reflect Vector Addition</v>
       </c>
       <c r="E176" t="str">
         <v>Model/UI defined</v>
@@ -10526,16 +10922,16 @@
     </row>
     <row r="177">
       <c r="A177" t="str">
-        <v>MAT-VEC-001</v>
+        <v>MAT-SEQ-001</v>
       </c>
       <c r="B177">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C177" t="str">
-        <v>REFLECT</v>
+        <v>OBSERVE</v>
       </c>
       <c r="D177" t="str">
-        <v>Reflect Vector Addition</v>
+        <v>Observe Sequences and Series</v>
       </c>
       <c r="E177" t="str">
         <v>Model/UI defined</v>
@@ -10546,13 +10942,13 @@
         <v>MAT-SEQ-001</v>
       </c>
       <c r="B178">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C178" t="str">
-        <v>OBSERVE</v>
+        <v>INTERACT</v>
       </c>
       <c r="D178" t="str">
-        <v>Observe Sequences and Series</v>
+        <v>Interact Sequences and Series</v>
       </c>
       <c r="E178" t="str">
         <v>Model/UI defined</v>
@@ -10563,13 +10959,13 @@
         <v>MAT-SEQ-001</v>
       </c>
       <c r="B179">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C179" t="str">
-        <v>INTERACT</v>
+        <v>MEASURE</v>
       </c>
       <c r="D179" t="str">
-        <v>Interact Sequences and Series</v>
+        <v>Measure Sequences and Series</v>
       </c>
       <c r="E179" t="str">
         <v>Model/UI defined</v>
@@ -10580,38 +10976,21 @@
         <v>MAT-SEQ-001</v>
       </c>
       <c r="B180">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C180" t="str">
-        <v>MEASURE</v>
+        <v>REFLECT</v>
       </c>
       <c r="D180" t="str">
-        <v>Measure Sequences and Series</v>
+        <v>Reflect Sequences and Series</v>
       </c>
       <c r="E180" t="str">
-        <v>Model/UI defined</v>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" t="str">
-        <v>MAT-SEQ-001</v>
-      </c>
-      <c r="B181">
-        <v>4</v>
-      </c>
-      <c r="C181" t="str">
-        <v>REFLECT</v>
-      </c>
-      <c r="D181" t="str">
-        <v>Reflect Sequences and Series</v>
-      </c>
-      <c r="E181" t="str">
         <v>Model/UI defined</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E181"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E180"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>